<commit_message>
KCPM-89 Test BVA với module Product #done
</commit_message>
<xml_diff>
--- a/automation/postman/VGA-store-product/VGA-store_product_AutoTest.xlsx
+++ b/automation/postman/VGA-store-product/VGA-store_product_AutoTest.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\bỏ tạm\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Kiểm chứng phần mềm\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ADCE0E6-A9F0-45AE-B428-A9E865321DBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABC9E590-0C36-4BEA-8A5B-46B597BDB107}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Product_TestCases" sheetId="5" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="567" uniqueCount="211">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="819" uniqueCount="288">
   <si>
     <t>VGA STORE – PRODUCT MODULE TEST CASES</t>
   </si>
@@ -670,6 +670,237 @@
   </si>
   <si>
     <t>📊 PRODUCT MODULE – TEST SUMMARY DASHBOARD</t>
+  </si>
+  <si>
+    <t>Lọc giá với minPrice bằng 0</t>
+  </si>
+  <si>
+    <t>Danh sách VGA hiển thị đúng khoảng giá, HTTP Code 200</t>
+  </si>
+  <si>
+    <t>TC_PROD_031</t>
+  </si>
+  <si>
+    <t>Lọc giá lỗi - minPrice là số âm</t>
+  </si>
+  <si>
+    <t>minPrice=-1500000</t>
+  </si>
+  <si>
+    <t>Hệ thống báo lỗi "Giá không được nhỏ hơn 0", HTTP Code 400</t>
+  </si>
+  <si>
+    <t>TC_PROD_032</t>
+  </si>
+  <si>
+    <t>Lọc giá lỗi - maxPrice là số âm</t>
+  </si>
+  <si>
+    <t>maxPrice=-5000000</t>
+  </si>
+  <si>
+    <t>TC_PROD_033</t>
+  </si>
+  <si>
+    <t>Lọc giá biên - logic minPrice lớn hơn maxPrice</t>
+  </si>
+  <si>
+    <t>Hệ thống báo lỗi khoảng giá không hợp lệ, HTTP Code 400</t>
+  </si>
+  <si>
+    <t>TC_PROD_034</t>
+  </si>
+  <si>
+    <t>Lọc giá biên - maxPrice bằng 0</t>
+  </si>
+  <si>
+    <t>Trả về danh sách rỗng hoặc sản phẩm giá 0đ, HTTP Code 200</t>
+  </si>
+  <si>
+    <t>TC_PROD_035</t>
+  </si>
+  <si>
+    <t>Lọc giá lỗi - minPrice bị tràn số (Overflow)</t>
+  </si>
+  <si>
+    <t>minPrice=9999999999999999</t>
+  </si>
+  <si>
+    <t>Hệ thống báo lỗi giá trị vượt quá giới hạn, HTTP Code 400</t>
+  </si>
+  <si>
+    <t>TC_PROD_036</t>
+  </si>
+  <si>
+    <t>Lọc giá lỗi - maxPrice bị tràn số (Overflow)</t>
+  </si>
+  <si>
+    <t>maxPrice=9999999999999999</t>
+  </si>
+  <si>
+    <t>TC_PROD_037</t>
+  </si>
+  <si>
+    <t>Phân trang lỗi - Số lượng trang (page) bằng 0</t>
+  </si>
+  <si>
+    <t>Hệ thống báo lỗi số trang không hợp lệ, HTTP Code 400</t>
+  </si>
+  <si>
+    <t>TC_PROD_038</t>
+  </si>
+  <si>
+    <t>Phân trang lỗi - Số lượng trang (page) là số âm</t>
+  </si>
+  <si>
+    <t>TC_PROD_039</t>
+  </si>
+  <si>
+    <t>Phân trang lỗi - Số lượng hiển thị (limit) bằng 0</t>
+  </si>
+  <si>
+    <t>Hệ thống báo lỗi kích thước trang không hợp lệ, HTTP Code 400</t>
+  </si>
+  <si>
+    <t>TC_PROD_040</t>
+  </si>
+  <si>
+    <t>Phân trang lỗi - Số lượng hiển thị (limit) âm</t>
+  </si>
+  <si>
+    <t>TC_PROD_041</t>
+  </si>
+  <si>
+    <t>minPrice=20000000, maxPrice=5000000</t>
+  </si>
+  <si>
+    <t>1. Chọn khoảng maxPrice bằng 0</t>
+  </si>
+  <si>
+    <t>minPrice=0, maxPrice=0</t>
+  </si>
+  <si>
+    <t>page=0, limit=10</t>
+  </si>
+  <si>
+    <t>page=-5, limit=10</t>
+  </si>
+  <si>
+    <t>page=1, limit=0</t>
+  </si>
+  <si>
+    <t>page=1, limit=-10</t>
+  </si>
+  <si>
+    <t>page=9999, limit=10</t>
+  </si>
+  <si>
+    <t>/api/products?minPrice=0&amp;maxPrice=20000000</t>
+  </si>
+  <si>
+    <t>products: [...]</t>
+  </si>
+  <si>
+    <t>/api/products?minPrice=-1500000</t>
+  </si>
+  <si>
+    <t>{"error": "Giá không được nhỏ hơn 0"}</t>
+  </si>
+  <si>
+    <t>/api/products?maxPrice=-5000000</t>
+  </si>
+  <si>
+    <t>/api/products?minPrice=20000000&amp;maxPrice=5000000</t>
+  </si>
+  <si>
+    <t>{"error": "Khoảng giá minPrice không được lớn hơn maxPrice"}</t>
+  </si>
+  <si>
+    <t>/api/products?minPrice=0&amp;maxPrice=0</t>
+  </si>
+  <si>
+    <t>/api/products?minPrice=9999999999999999</t>
+  </si>
+  <si>
+    <t>{"error": "Giá trị vượt quá giới hạn cho phép (Overflow)"}</t>
+  </si>
+  <si>
+    <t>/api/products?maxPrice=9999999999999999</t>
+  </si>
+  <si>
+    <t>/api/products?page=0&amp;limit=10</t>
+  </si>
+  <si>
+    <t>{"error": "Số trang phải lớn hơn hoặc bằng 1"}</t>
+  </si>
+  <si>
+    <t>/api/products?page=-5&amp;limit=10</t>
+  </si>
+  <si>
+    <t>/api/products?page=1&amp;limit=0</t>
+  </si>
+  <si>
+    <t>{"error": "Số lượng hiển thị phải lớn hơn hoặc bằng 1"}</t>
+  </si>
+  <si>
+    <t>/api/products?page=1&amp;limit=-10</t>
+  </si>
+  <si>
+    <t>/api/products?page=9999&amp;limit=10</t>
+  </si>
+  <si>
+    <t>{"currentPage": 9999, "products": []}</t>
+  </si>
+  <si>
+    <t>{"currentPage": 1, "products": []}</t>
+  </si>
+  <si>
+    <t>TC_PROD_042</t>
+  </si>
+  <si>
+    <t>Người dùng truy cập danh mục sản phẩm</t>
+  </si>
+  <si>
+    <t>1. Chọn khoảng giá minPrice bằng 0</t>
+  </si>
+  <si>
+    <t>1. Nhập khoảng minPrice mang giá trị âm</t>
+  </si>
+  <si>
+    <t>1. Nhập khoảng maxPrice mang giá trị âm</t>
+  </si>
+  <si>
+    <t>1. Nhập giá trị minPrice lớn hơn maxPrice</t>
+  </si>
+  <si>
+    <t>1. Nhập giá trị minPrice vượt giới hạn lưu trữ</t>
+  </si>
+  <si>
+    <t>1. Nhập giá trị maxPrice vượt giới hạn lưu trữ</t>
+  </si>
+  <si>
+    <t>1. Nhập tham số số trang page bằng 0</t>
+  </si>
+  <si>
+    <t>1. Nhập tham số số trang page mang giá trị âm</t>
+  </si>
+  <si>
+    <t>1. Nhập số lượng hiển thị limit bằng 0</t>
+  </si>
+  <si>
+    <t>1. Nhập số lượng hiển thị limit mang giá trị âm</t>
+  </si>
+  <si>
+    <t>Phân trang biên - Số trang vượt quá dữ liệu</t>
+  </si>
+  <si>
+    <t>1. Nhập số trang page cực lớn vượt dữ liệu hiện tại</t>
+  </si>
+  <si>
+    <t>minPrice=0, maxPrice=20000000</t>
+  </si>
+  <si>
+    <t>Trả về mảng rỗng [] hoặc trang rỗng, HTTP Code 200</t>
   </si>
 </sst>
 </file>
@@ -677,9 +908,9 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="168" formatCode="0.0&quot;%&quot;"/>
+    <numFmt numFmtId="164" formatCode="0.0&quot;%&quot;"/>
   </numFmts>
-  <fonts count="15" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -786,6 +1017,21 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF1F1F1F"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -877,11 +1123,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -942,12 +1185,27 @@
     <xf numFmtId="0" fontId="1" fillId="12" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="168" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="12" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment readingOrder="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1229,943 +1487,1365 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7B9FB171-A3AA-463B-838F-EDC01E820D15}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K39"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="3" max="3" width="23.88671875" customWidth="1"/>
-    <col min="4" max="4" width="22.5546875" customWidth="1"/>
-    <col min="5" max="5" width="43.109375" customWidth="1"/>
-    <col min="6" max="6" width="40.77734375" customWidth="1"/>
-    <col min="7" max="7" width="40.6640625" customWidth="1"/>
-    <col min="8" max="8" width="30.88671875" customWidth="1"/>
-    <col min="9" max="9" width="69.109375" customWidth="1"/>
-    <col min="10" max="10" width="11.6640625" customWidth="1"/>
-    <col min="11" max="11" width="9.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.6640625" style="25" customWidth="1"/>
+    <col min="2" max="2" width="8.88671875" style="25"/>
+    <col min="3" max="3" width="23.88671875" style="25" customWidth="1"/>
+    <col min="4" max="4" width="22.5546875" style="25" customWidth="1"/>
+    <col min="5" max="5" width="43.109375" style="25" customWidth="1"/>
+    <col min="6" max="6" width="40.77734375" style="25" customWidth="1"/>
+    <col min="7" max="7" width="40.6640625" style="25" customWidth="1"/>
+    <col min="8" max="8" width="30.88671875" style="25" customWidth="1"/>
+    <col min="9" max="9" width="69.109375" style="25" customWidth="1"/>
+    <col min="10" max="10" width="11.6640625" style="25" customWidth="1"/>
+    <col min="11" max="11" width="9.44140625" style="25" customWidth="1"/>
+    <col min="12" max="16384" width="8.88671875" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
-      <c r="J1" s="1"/>
-      <c r="K1" s="1"/>
+      <c r="B1" s="24"/>
+      <c r="C1" s="24"/>
+      <c r="D1" s="24"/>
+      <c r="E1" s="24"/>
+      <c r="F1" s="24"/>
+      <c r="G1" s="24"/>
+      <c r="H1" s="24"/>
+      <c r="I1" s="24"/>
+      <c r="J1" s="24"/>
+      <c r="K1" s="24"/>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="26" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="C2" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="26" t="s">
         <v>4</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="26" t="s">
         <v>5</v>
       </c>
-      <c r="F2" t="s">
+      <c r="F2" s="26" t="s">
         <v>6</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="H2" t="s">
+      <c r="H2" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="I2" t="s">
+      <c r="I2" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="J2" t="s">
+      <c r="J2" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="K2" t="s">
+      <c r="K2" s="26" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="26" t="s">
         <v>12</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C3" t="s">
-        <v>14</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="C3" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D3" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="F3" t="s">
+      <c r="F3" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="H3" t="s">
+      <c r="H3" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="I3" t="s">
+      <c r="I3" s="26" t="s">
         <v>149</v>
       </c>
-      <c r="J3" t="s">
+      <c r="J3" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K3" t="s">
+      <c r="K3" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="26" t="s">
         <v>20</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C4" t="s">
-        <v>14</v>
-      </c>
-      <c r="D4" t="s">
+      <c r="C4" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D4" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="26" t="s">
         <v>21</v>
       </c>
-      <c r="F4" t="s">
+      <c r="F4" s="26" t="s">
         <v>22</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="H4" t="s">
+      <c r="H4" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="I4" t="s">
+      <c r="I4" s="26" t="s">
         <v>24</v>
       </c>
-      <c r="J4" t="s">
+      <c r="J4" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K4" t="s">
+      <c r="K4" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="26" t="s">
         <v>26</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C5" t="s">
-        <v>14</v>
-      </c>
-      <c r="D5" t="s">
+      <c r="C5" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="26" t="s">
         <v>27</v>
       </c>
-      <c r="F5" t="s">
+      <c r="F5" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="H5" t="s">
+      <c r="H5" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="I5" t="s">
+      <c r="I5" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="J5" t="s">
+      <c r="J5" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K5" t="s">
+      <c r="K5" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C6" t="s">
-        <v>14</v>
-      </c>
-      <c r="D6" t="s">
+      <c r="C6" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D6" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="26" t="s">
         <v>30</v>
       </c>
-      <c r="F6" t="s">
+      <c r="F6" s="26" t="s">
         <v>31</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="H6" t="s">
+      <c r="H6" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="I6" t="s">
+      <c r="I6" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="J6" t="s">
+      <c r="J6" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K6" t="s">
+      <c r="K6" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="26" t="s">
         <v>32</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B7" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" t="s">
+      <c r="C7" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D7" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="26" t="s">
         <v>33</v>
       </c>
-      <c r="F7" t="s">
+      <c r="F7" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="H7" t="s">
+      <c r="H7" s="26" t="s">
         <v>23</v>
       </c>
-      <c r="I7" t="s">
+      <c r="I7" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="J7" t="s">
+      <c r="J7" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="K7" t="s">
+      <c r="K7" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B8" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C8" t="s">
-        <v>14</v>
-      </c>
-      <c r="D8" t="s">
+      <c r="C8" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D8" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="F8" t="s">
+      <c r="F8" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="H8" t="s">
+      <c r="H8" s="26" t="s">
         <v>150</v>
       </c>
-      <c r="I8" t="s">
+      <c r="I8" s="26" t="s">
         <v>200</v>
       </c>
-      <c r="J8" t="s">
+      <c r="J8" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="26" t="s">
         <v>39</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C9" t="s">
-        <v>14</v>
-      </c>
-      <c r="D9" t="s">
+      <c r="C9" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D9" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="26" t="s">
         <v>40</v>
       </c>
-      <c r="F9" t="s">
+      <c r="F9" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="26" t="s">
         <v>86</v>
       </c>
-      <c r="H9" t="s">
+      <c r="H9" s="26" t="s">
         <v>151</v>
       </c>
-      <c r="I9" t="s">
+      <c r="I9" s="26" t="s">
         <v>201</v>
       </c>
-      <c r="J9" t="s">
+      <c r="J9" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K9" t="s">
+      <c r="K9" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C10" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" t="s">
+      <c r="C10" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D10" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="F10" t="s">
+      <c r="F10" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="H10" t="s">
+      <c r="H10" s="26" t="s">
         <v>45</v>
       </c>
-      <c r="I10" t="s">
+      <c r="I10" s="26" t="s">
         <v>46</v>
       </c>
-      <c r="J10" t="s">
+      <c r="J10" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K10" t="s">
+      <c r="K10" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="26" t="s">
         <v>47</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C11" t="s">
-        <v>14</v>
-      </c>
-      <c r="D11" t="s">
+      <c r="C11" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D11" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="26" t="s">
         <v>48</v>
       </c>
-      <c r="F11" t="s">
+      <c r="F11" s="26" t="s">
         <v>44</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="H11" t="s">
+      <c r="H11" s="26" t="s">
         <v>49</v>
       </c>
-      <c r="I11" t="s">
+      <c r="I11" s="26" t="s">
         <v>50</v>
       </c>
-      <c r="J11" t="s">
+      <c r="J11" s="26" t="s">
         <v>36</v>
       </c>
-      <c r="K11" t="s">
+      <c r="K11" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="26" t="s">
         <v>51</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C12" t="s">
-        <v>14</v>
-      </c>
-      <c r="D12" t="s">
+      <c r="C12" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D12" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="26" t="s">
         <v>52</v>
       </c>
-      <c r="F12" t="s">
+      <c r="F12" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="H12" t="s">
+      <c r="H12" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="I12" t="s">
+      <c r="I12" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="J12" t="s">
+      <c r="J12" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K12" t="s">
+      <c r="K12" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="26" t="s">
         <v>54</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C13" t="s">
-        <v>14</v>
-      </c>
-      <c r="D13" t="s">
+      <c r="C13" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D13" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="26" t="s">
         <v>55</v>
       </c>
-      <c r="F13" t="s">
+      <c r="F13" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="26" t="s">
         <v>92</v>
       </c>
-      <c r="H13" t="s">
+      <c r="H13" s="26" t="s">
         <v>56</v>
       </c>
-      <c r="I13" t="s">
+      <c r="I13" s="26" t="s">
         <v>93</v>
       </c>
-      <c r="J13" t="s">
+      <c r="J13" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K13" t="s">
+      <c r="K13" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="26" t="s">
         <v>57</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C14" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14" t="s">
+      <c r="C14" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D14" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="26" t="s">
         <v>58</v>
       </c>
-      <c r="F14" t="s">
+      <c r="F14" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="H14" t="s">
+      <c r="H14" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="I14" t="s">
+      <c r="I14" s="26" t="s">
         <v>96</v>
       </c>
-      <c r="J14" t="s">
+      <c r="J14" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K14" t="s">
+      <c r="K14" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C15" t="s">
-        <v>14</v>
-      </c>
-      <c r="D15" t="s">
+      <c r="C15" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D15" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F15" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="H15" t="s">
+      <c r="H15" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I15" s="26" t="s">
         <v>99</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J15" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K15" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C16" t="s">
-        <v>14</v>
-      </c>
-      <c r="D16" t="s">
+      <c r="C16" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D16" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F16" s="26" t="s">
         <v>100</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="26" t="s">
         <v>101</v>
       </c>
-      <c r="H16" t="s">
+      <c r="H16" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I16" s="26" t="s">
         <v>202</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J16" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K16" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C17" t="s">
-        <v>14</v>
-      </c>
-      <c r="D17" t="s">
+      <c r="C17" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D17" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F17" s="26" t="s">
         <v>102</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="26" t="s">
         <v>103</v>
       </c>
-      <c r="H17" t="s">
+      <c r="H17" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I17" s="26" t="s">
         <v>104</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J17" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K17" t="s">
+      <c r="K17" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="26" t="s">
         <v>68</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C18" t="s">
-        <v>14</v>
-      </c>
-      <c r="D18" t="s">
+      <c r="C18" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D18" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F18" s="26" t="s">
         <v>105</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="H18" t="s">
+      <c r="H18" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I18" s="26" t="s">
         <v>107</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J18" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K18" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="19" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="A19" s="26" t="s">
         <v>71</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C19" t="s">
-        <v>14</v>
-      </c>
-      <c r="D19" t="s">
+      <c r="C19" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D19" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="26" t="s">
         <v>72</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F19" s="26" t="s">
         <v>108</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="H19" t="s">
+      <c r="H19" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I19" s="26" t="s">
         <v>109</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J19" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K19" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="20" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="A20" s="26" t="s">
         <v>110</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C20" t="s">
-        <v>14</v>
-      </c>
-      <c r="D20" t="s">
+      <c r="C20" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D20" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="26" t="s">
         <v>111</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F20" s="26" t="s">
         <v>89</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="26" t="s">
         <v>106</v>
       </c>
-      <c r="H20" t="s">
+      <c r="H20" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I20" s="26" t="s">
         <v>112</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J20" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K20" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="21" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="26" t="s">
         <v>113</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C21" t="s">
-        <v>14</v>
-      </c>
-      <c r="D21" t="s">
+      <c r="C21" s="26" t="s">
+        <v>14</v>
+      </c>
+      <c r="D21" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="26" t="s">
         <v>114</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F21" s="26" t="s">
         <v>115</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="26" t="s">
         <v>116</v>
       </c>
-      <c r="H21" t="s">
+      <c r="H21" s="26" t="s">
         <v>117</v>
       </c>
-      <c r="I21" t="s">
+      <c r="I21" s="26" t="s">
         <v>152</v>
       </c>
-      <c r="J21" t="s">
+      <c r="J21" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K21" t="s">
+      <c r="K21" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="22" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="A22" s="26" t="s">
         <v>118</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="26" t="s">
         <v>120</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F22" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="26" t="s">
         <v>122</v>
       </c>
-      <c r="H22" t="s">
+      <c r="H22" s="26" t="s">
         <v>123</v>
       </c>
-      <c r="I22" t="s">
+      <c r="I22" s="26" t="s">
         <v>124</v>
       </c>
-      <c r="J22" t="s">
+      <c r="J22" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K22" t="s">
+      <c r="K22" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="23" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="A23" s="26" t="s">
         <v>125</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="26" t="s">
         <v>119</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="26" t="s">
         <v>126</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F23" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="26" t="s">
         <v>153</v>
       </c>
-      <c r="H23" t="s">
+      <c r="H23" s="26" t="s">
         <v>154</v>
       </c>
-      <c r="I23" t="s">
+      <c r="I23" s="26" t="s">
         <v>127</v>
       </c>
-      <c r="J23" t="s">
+      <c r="J23" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K23" t="s">
+      <c r="K23" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="24" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="A24" s="26" t="s">
         <v>128</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="26" t="s">
         <v>129</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="26" t="s">
         <v>130</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F24" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="26" t="s">
         <v>132</v>
       </c>
-      <c r="H24" t="s">
+      <c r="H24" s="26" t="s">
         <v>155</v>
       </c>
-      <c r="I24" t="s">
+      <c r="I24" s="26" t="s">
         <v>133</v>
       </c>
-      <c r="J24" t="s">
+      <c r="J24" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K24" t="s">
+      <c r="K24" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="25" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="A25" s="26" t="s">
         <v>134</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="26" t="s">
         <v>129</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="26" t="s">
         <v>135</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F25" s="26" t="s">
         <v>121</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="26" t="s">
         <v>136</v>
       </c>
-      <c r="H25" t="s">
+      <c r="H25" s="26" t="s">
         <v>156</v>
       </c>
-      <c r="I25" t="s">
+      <c r="I25" s="26" t="s">
         <v>137</v>
       </c>
-      <c r="J25" t="s">
+      <c r="J25" s="26" t="s">
         <v>25</v>
       </c>
-      <c r="K25" t="s">
+      <c r="K25" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="26" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="A26" s="26" t="s">
         <v>138</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="26" t="s">
         <v>140</v>
       </c>
-      <c r="F26" t="s">
+      <c r="F26" s="26" t="s">
         <v>131</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="26" t="s">
         <v>141</v>
       </c>
-      <c r="H26" t="s">
+      <c r="H26" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="I26" t="s">
+      <c r="I26" s="26" t="s">
         <v>157</v>
       </c>
-      <c r="J26" t="s">
+      <c r="J26" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K26" t="s">
+      <c r="K26" s="26" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="27" spans="1:11" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
+      <c r="A27" s="26" t="s">
         <v>142</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="26" t="s">
         <v>139</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="26" t="s">
         <v>143</v>
       </c>
-      <c r="F27" t="s">
+      <c r="F27" s="26" t="s">
         <v>144</v>
       </c>
-      <c r="G27" t="s">
+      <c r="G27" s="26" t="s">
         <v>145</v>
       </c>
-      <c r="H27" t="s">
+      <c r="H27" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="I27" t="s">
+      <c r="I27" s="26" t="s">
         <v>146</v>
       </c>
-      <c r="J27" t="s">
+      <c r="J27" s="26" t="s">
         <v>18</v>
       </c>
-      <c r="K27" t="s">
+      <c r="K27" s="26" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A28" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E28" s="27" t="s">
+        <v>211</v>
+      </c>
+      <c r="F28" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G28" s="27" t="s">
+        <v>274</v>
+      </c>
+      <c r="H28" s="27" t="s">
+        <v>286</v>
+      </c>
+      <c r="I28" s="27" t="s">
+        <v>212</v>
+      </c>
+      <c r="J28" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K28" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A29" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E29" s="27" t="s">
+        <v>214</v>
+      </c>
+      <c r="F29" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G29" s="27" t="s">
+        <v>275</v>
+      </c>
+      <c r="H29" s="27" t="s">
+        <v>215</v>
+      </c>
+      <c r="I29" s="27" t="s">
+        <v>216</v>
+      </c>
+      <c r="J29" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K29" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A30" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E30" s="27" t="s">
+        <v>218</v>
+      </c>
+      <c r="F30" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>276</v>
+      </c>
+      <c r="H30" s="27" t="s">
+        <v>219</v>
+      </c>
+      <c r="I30" s="27" t="s">
+        <v>216</v>
+      </c>
+      <c r="J30" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K30" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A31" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E31" s="27" t="s">
+        <v>221</v>
+      </c>
+      <c r="F31" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G31" s="27" t="s">
+        <v>277</v>
+      </c>
+      <c r="H31" s="27" t="s">
+        <v>244</v>
+      </c>
+      <c r="I31" s="27" t="s">
+        <v>222</v>
+      </c>
+      <c r="J31" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K31" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A32" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E32" s="27" t="s">
+        <v>224</v>
+      </c>
+      <c r="F32" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G32" s="27" t="s">
+        <v>245</v>
+      </c>
+      <c r="H32" s="27" t="s">
+        <v>246</v>
+      </c>
+      <c r="I32" s="27" t="s">
+        <v>225</v>
+      </c>
+      <c r="J32" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="K32" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A33" s="27" t="s">
+        <v>230</v>
+      </c>
+      <c r="B33" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C33" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E33" s="27" t="s">
+        <v>227</v>
+      </c>
+      <c r="F33" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G33" s="27" t="s">
+        <v>278</v>
+      </c>
+      <c r="H33" s="27" t="s">
+        <v>228</v>
+      </c>
+      <c r="I33" s="27" t="s">
+        <v>229</v>
+      </c>
+      <c r="J33" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K33" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="34" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A34" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="B34" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E34" s="27" t="s">
+        <v>231</v>
+      </c>
+      <c r="F34" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G34" s="27" t="s">
+        <v>279</v>
+      </c>
+      <c r="H34" s="27" t="s">
+        <v>232</v>
+      </c>
+      <c r="I34" s="27" t="s">
+        <v>229</v>
+      </c>
+      <c r="J34" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K34" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="35" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A35" s="27" t="s">
+        <v>236</v>
+      </c>
+      <c r="B35" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E35" s="27" t="s">
+        <v>234</v>
+      </c>
+      <c r="F35" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G35" s="27" t="s">
+        <v>280</v>
+      </c>
+      <c r="H35" s="27" t="s">
+        <v>247</v>
+      </c>
+      <c r="I35" s="27" t="s">
+        <v>235</v>
+      </c>
+      <c r="J35" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K35" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="36" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A36" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E36" s="27" t="s">
+        <v>237</v>
+      </c>
+      <c r="F36" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G36" s="27" t="s">
+        <v>281</v>
+      </c>
+      <c r="H36" s="27" t="s">
+        <v>248</v>
+      </c>
+      <c r="I36" s="27" t="s">
+        <v>235</v>
+      </c>
+      <c r="J36" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K36" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="37" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A37" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="B37" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E37" s="27" t="s">
+        <v>239</v>
+      </c>
+      <c r="F37" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G37" s="27" t="s">
+        <v>282</v>
+      </c>
+      <c r="H37" s="27" t="s">
+        <v>249</v>
+      </c>
+      <c r="I37" s="27" t="s">
+        <v>240</v>
+      </c>
+      <c r="J37" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K37" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="38" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A38" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C38" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E38" s="27" t="s">
+        <v>242</v>
+      </c>
+      <c r="F38" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G38" s="27" t="s">
+        <v>283</v>
+      </c>
+      <c r="H38" s="27" t="s">
+        <v>250</v>
+      </c>
+      <c r="I38" s="27" t="s">
+        <v>240</v>
+      </c>
+      <c r="J38" s="27" t="s">
+        <v>18</v>
+      </c>
+      <c r="K38" s="27" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="39" spans="1:11" x14ac:dyDescent="0.3">
+      <c r="A39" s="27" t="s">
+        <v>272</v>
+      </c>
+      <c r="B39" s="27" t="s">
+        <v>13</v>
+      </c>
+      <c r="C39" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="D39" s="27" t="s">
+        <v>15</v>
+      </c>
+      <c r="E39" s="27" t="s">
+        <v>284</v>
+      </c>
+      <c r="F39" s="27" t="s">
+        <v>273</v>
+      </c>
+      <c r="G39" s="27" t="s">
+        <v>285</v>
+      </c>
+      <c r="H39" s="27" t="s">
+        <v>251</v>
+      </c>
+      <c r="I39" s="27" t="s">
+        <v>287</v>
+      </c>
+      <c r="J39" s="27" t="s">
+        <v>25</v>
+      </c>
+      <c r="K39" s="27" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2179,614 +2859,891 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEF9B249-1455-4465-8888-A946B8483E8D}">
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="30.44140625" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
-    <col min="3" max="3" width="64.77734375" customWidth="1"/>
-    <col min="4" max="4" width="64.88671875" customWidth="1"/>
-    <col min="5" max="5" width="53.6640625" customWidth="1"/>
-    <col min="6" max="6" width="17.77734375" customWidth="1"/>
-    <col min="7" max="7" width="33.88671875" customWidth="1"/>
+    <col min="1" max="1" width="15.109375" style="25" customWidth="1"/>
+    <col min="2" max="2" width="12.6640625" style="25" customWidth="1"/>
+    <col min="3" max="3" width="58.44140625" style="25" customWidth="1"/>
+    <col min="4" max="4" width="59.77734375" style="25" customWidth="1"/>
+    <col min="5" max="5" width="53.6640625" style="25" customWidth="1"/>
+    <col min="6" max="6" width="17.77734375" style="25" customWidth="1"/>
+    <col min="7" max="7" width="33.88671875" style="25" customWidth="1"/>
+    <col min="8" max="16384" width="8.88671875" style="25"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="29" t="s">
         <v>4</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="29" t="s">
         <v>158</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="29" t="s">
         <v>159</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="29" t="s">
         <v>160</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="29" t="s">
         <v>161</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="A2" s="29" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
-        <v>14</v>
-      </c>
-      <c r="C2" t="s">
+      <c r="B2" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C2" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E2" t="s">
+      <c r="E2" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="29">
         <v>200</v>
       </c>
-      <c r="G2" t="s">
+      <c r="G2" s="29" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+      <c r="A3" s="29" t="s">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="B3" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D3" t="s">
+      <c r="D3" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="29">
         <v>200</v>
       </c>
-      <c r="G3" t="s">
+      <c r="G3" s="29" t="s">
         <v>165</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+      <c r="A4" s="29" t="s">
         <v>26</v>
       </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="B4" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D4" t="s">
+      <c r="D4" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="29">
         <v>200</v>
       </c>
-      <c r="G4" t="s">
+      <c r="G4" s="29" t="s">
         <v>166</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" t="s">
+      <c r="A5" s="29" t="s">
         <v>29</v>
       </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="B5" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D5" t="s">
+      <c r="D5" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="29">
         <v>200</v>
       </c>
-      <c r="G5" t="s">
+      <c r="G5" s="29" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
+      <c r="A6" s="29" t="s">
         <v>32</v>
       </c>
-      <c r="B6" t="s">
-        <v>14</v>
-      </c>
-      <c r="C6" t="s">
+      <c r="B6" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C6" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="29">
         <v>200</v>
       </c>
-      <c r="G6" t="s">
+      <c r="G6" s="29" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
+      <c r="A7" s="29" t="s">
         <v>37</v>
       </c>
-      <c r="B7" t="s">
-        <v>14</v>
-      </c>
-      <c r="C7" t="s">
+      <c r="B7" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="29" t="s">
         <v>169</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E7" t="s">
+      <c r="E7" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F7">
+      <c r="F7" s="29">
         <v>200</v>
       </c>
-      <c r="G7" t="s">
+      <c r="G7" s="29" t="s">
         <v>170</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
+      <c r="A8" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="B8" t="s">
-        <v>14</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B8" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="29" t="s">
         <v>171</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="29">
         <v>200</v>
       </c>
-      <c r="G8" t="s">
+      <c r="G8" s="29" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" t="s">
+      <c r="A9" s="29" t="s">
         <v>42</v>
       </c>
-      <c r="B9" t="s">
-        <v>14</v>
-      </c>
-      <c r="C9" t="s">
+      <c r="B9" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C9" s="29" t="s">
         <v>173</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F9">
+      <c r="F9" s="29">
         <v>200</v>
       </c>
-      <c r="G9" t="s">
+      <c r="G9" s="29" t="s">
         <v>174</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" t="s">
+      <c r="A10" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="B10" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="B10" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C10" s="29" t="s">
         <v>175</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="29">
         <v>200</v>
       </c>
-      <c r="G10" t="s">
+      <c r="G10" s="29" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" t="s">
+      <c r="A11" s="29" t="s">
         <v>51</v>
       </c>
-      <c r="B11" t="s">
-        <v>14</v>
-      </c>
-      <c r="C11" t="s">
+      <c r="B11" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C11" s="29" t="s">
         <v>176</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="29">
         <v>200</v>
       </c>
-      <c r="G11" t="s">
+      <c r="G11" s="29" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" t="s">
+      <c r="A12" s="29" t="s">
         <v>54</v>
       </c>
-      <c r="B12" t="s">
-        <v>14</v>
-      </c>
-      <c r="C12" t="s">
+      <c r="B12" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" s="29" t="s">
         <v>177</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="29">
         <v>200</v>
       </c>
-      <c r="G12" t="s">
+      <c r="G12" s="29" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" t="s">
+      <c r="A13" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="B13" t="s">
-        <v>14</v>
-      </c>
-      <c r="C13" t="s">
+      <c r="B13" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C13" s="29" t="s">
         <v>178</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="29">
         <v>200</v>
       </c>
-      <c r="G13" t="s">
+      <c r="G13" s="29" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" t="s">
+      <c r="A14" s="29" t="s">
         <v>60</v>
       </c>
-      <c r="B14" t="s">
-        <v>14</v>
-      </c>
-      <c r="C14" t="s">
+      <c r="B14" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C14" s="29" t="s">
         <v>180</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="29">
         <v>200</v>
       </c>
-      <c r="G14" t="s">
+      <c r="G14" s="29" t="s">
         <v>181</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
+      <c r="A15" s="29" t="s">
         <v>63</v>
       </c>
-      <c r="B15" t="s">
-        <v>14</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="B15" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C15" s="29" t="s">
         <v>182</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E15" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="29">
         <v>200</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G15" s="29" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" t="s">
+      <c r="A16" s="29" t="s">
         <v>65</v>
       </c>
-      <c r="B16" t="s">
-        <v>14</v>
-      </c>
-      <c r="C16" t="s">
+      <c r="B16" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C16" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="29">
         <v>200</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G16" s="29" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A17" t="s">
+      <c r="A17" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="B17" t="s">
-        <v>14</v>
-      </c>
-      <c r="C17" t="s">
+      <c r="B17" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="29">
         <v>200</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G17" s="29" t="s">
         <v>185</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A18" t="s">
+      <c r="A18" s="29" t="s">
         <v>71</v>
       </c>
-      <c r="B18" t="s">
-        <v>14</v>
-      </c>
-      <c r="C18" t="s">
+      <c r="B18" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="29">
         <v>200</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G18" s="29" t="s">
         <v>186</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" t="s">
+      <c r="A19" s="29" t="s">
         <v>110</v>
       </c>
-      <c r="B19" t="s">
-        <v>14</v>
-      </c>
-      <c r="C19" t="s">
+      <c r="B19" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="29">
         <v>200</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G19" s="29" t="s">
         <v>167</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" t="s">
+      <c r="A20" s="29" t="s">
         <v>113</v>
       </c>
-      <c r="B20" t="s">
-        <v>14</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="B20" s="29" t="s">
+        <v>14</v>
+      </c>
+      <c r="C20" s="29" t="s">
         <v>187</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="29" t="s">
         <v>162</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="29">
         <v>404</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G20" s="29" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" t="s">
+      <c r="A21" s="29" t="s">
         <v>118</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="29" t="s">
         <v>189</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="29" t="s">
         <v>190</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="29">
         <v>201</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G21" s="29" t="s">
         <v>191</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A22" t="s">
+      <c r="A22" s="29" t="s">
         <v>125</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="29" t="s">
         <v>119</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="29" t="s">
         <v>15</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="29" t="s">
         <v>189</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="29" t="s">
         <v>192</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="29">
         <v>400</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G22" s="29" t="s">
         <v>193</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A23" t="s">
+      <c r="A23" s="29" t="s">
         <v>128</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="29" t="s">
         <v>129</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="29" t="s">
         <v>189</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="29" t="s">
         <v>194</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="29">
         <v>200</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G23" s="29" t="s">
         <v>195</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A24" t="s">
+      <c r="A24" s="29" t="s">
         <v>134</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="29" t="s">
         <v>129</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="29" t="s">
         <v>187</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="29" t="s">
         <v>189</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="29" t="s">
         <v>194</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="29">
         <v>404</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G24" s="29" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A25" t="s">
+      <c r="A25" s="29" t="s">
         <v>138</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="29" t="s">
         <v>196</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="29">
         <v>200</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G25" s="29" t="s">
         <v>197</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A26" t="s">
+      <c r="A26" s="29" t="s">
         <v>142</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="29" t="s">
         <v>139</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="29" t="s">
         <v>183</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="29" t="s">
         <v>198</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="29" t="s">
         <v>163</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="29">
         <v>403</v>
       </c>
-      <c r="G26" t="s">
+      <c r="G26" s="29" t="s">
         <v>199</v>
+      </c>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27" s="27" t="s">
+        <v>213</v>
+      </c>
+      <c r="B27" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C27" s="27" t="s">
+        <v>252</v>
+      </c>
+      <c r="D27" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E27" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F27" s="27">
+        <v>200</v>
+      </c>
+      <c r="G27" s="27" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28" s="27" t="s">
+        <v>217</v>
+      </c>
+      <c r="B28" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C28" s="27" t="s">
+        <v>254</v>
+      </c>
+      <c r="D28" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E28" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F28" s="27">
+        <v>400</v>
+      </c>
+      <c r="G28" s="27" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="29" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A29" s="27" t="s">
+        <v>220</v>
+      </c>
+      <c r="B29" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C29" s="27" t="s">
+        <v>256</v>
+      </c>
+      <c r="D29" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E29" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F29" s="27">
+        <v>400</v>
+      </c>
+      <c r="G29" s="27" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="30" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A30" s="27" t="s">
+        <v>223</v>
+      </c>
+      <c r="B30" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C30" s="27" t="s">
+        <v>257</v>
+      </c>
+      <c r="D30" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E30" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F30" s="27">
+        <v>400</v>
+      </c>
+      <c r="G30" s="27" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="31" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A31" s="27" t="s">
+        <v>226</v>
+      </c>
+      <c r="B31" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C31" s="27" t="s">
+        <v>259</v>
+      </c>
+      <c r="D31" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E31" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F31" s="27">
+        <v>200</v>
+      </c>
+      <c r="G31" s="27" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="32" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A32" s="27" t="s">
+        <v>230</v>
+      </c>
+      <c r="B32" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C32" s="27" t="s">
+        <v>260</v>
+      </c>
+      <c r="D32" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E32" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F32" s="27">
+        <v>400</v>
+      </c>
+      <c r="G32" s="27" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A33" s="27" t="s">
+        <v>233</v>
+      </c>
+      <c r="B33" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C33" s="27" t="s">
+        <v>262</v>
+      </c>
+      <c r="D33" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E33" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F33" s="27">
+        <v>400</v>
+      </c>
+      <c r="G33" s="27" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A34" s="27" t="s">
+        <v>236</v>
+      </c>
+      <c r="B34" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C34" s="27" t="s">
+        <v>263</v>
+      </c>
+      <c r="D34" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E34" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F34" s="27">
+        <v>400</v>
+      </c>
+      <c r="G34" s="27" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A35" s="27" t="s">
+        <v>238</v>
+      </c>
+      <c r="B35" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C35" s="27" t="s">
+        <v>265</v>
+      </c>
+      <c r="D35" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E35" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F35" s="27">
+        <v>400</v>
+      </c>
+      <c r="G35" s="27" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A36" s="27" t="s">
+        <v>241</v>
+      </c>
+      <c r="B36" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C36" s="27" t="s">
+        <v>266</v>
+      </c>
+      <c r="D36" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E36" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F36" s="27">
+        <v>400</v>
+      </c>
+      <c r="G36" s="27" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A37" s="27" t="s">
+        <v>243</v>
+      </c>
+      <c r="B37" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C37" s="27" t="s">
+        <v>268</v>
+      </c>
+      <c r="D37" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E37" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F37" s="27">
+        <v>400</v>
+      </c>
+      <c r="G37" s="27" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A38" s="27" t="s">
+        <v>272</v>
+      </c>
+      <c r="B38" s="27" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="27" t="s">
+        <v>269</v>
+      </c>
+      <c r="D38" s="27" t="s">
+        <v>162</v>
+      </c>
+      <c r="E38" s="28" t="s">
+        <v>163</v>
+      </c>
+      <c r="F38" s="27">
+        <v>200</v>
+      </c>
+      <c r="G38" s="27" t="s">
+        <v>270</v>
       </c>
     </row>
   </sheetData>
@@ -2796,12 +3753,15 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5A6C63D4-393A-4871-AE63-6C3C278E275A}">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="24.109375" customWidth="1"/>
     <col min="2" max="2" width="38.44140625" customWidth="1"/>
-    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="3" max="3" width="11.5546875" customWidth="1"/>
+    <col min="4" max="4" width="21.44140625" customWidth="1"/>
+    <col min="5" max="5" width="22" customWidth="1"/>
+    <col min="6" max="6" width="18.44140625" customWidth="1"/>
     <col min="7" max="7" width="24.44140625" customWidth="1"/>
     <col min="10" max="10" width="15.21875" customWidth="1"/>
   </cols>
@@ -3093,7 +4053,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>68</v>
       </c>
@@ -3110,7 +4070,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>71</v>
       </c>
@@ -3127,7 +4087,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>110</v>
       </c>
@@ -3144,7 +4104,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>113</v>
       </c>
@@ -3161,7 +4121,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>118</v>
       </c>
@@ -3178,7 +4138,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>125</v>
       </c>
@@ -3195,7 +4155,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>128</v>
       </c>
@@ -3212,7 +4172,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>134</v>
       </c>
@@ -3229,7 +4189,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>138</v>
       </c>
@@ -3246,7 +4206,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="26" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>142</v>
       </c>
@@ -3262,6 +4222,270 @@
       <c r="H26" t="s">
         <v>19</v>
       </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A27" s="30" t="s">
+        <v>213</v>
+      </c>
+      <c r="B27" s="30" t="s">
+        <v>211</v>
+      </c>
+      <c r="C27" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D27" s="30">
+        <v>200</v>
+      </c>
+      <c r="E27" s="30"/>
+      <c r="F27" s="30"/>
+      <c r="G27" s="30"/>
+      <c r="H27" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I27" s="30"/>
+      <c r="J27" s="30"/>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A28" s="30" t="s">
+        <v>217</v>
+      </c>
+      <c r="B28" s="30" t="s">
+        <v>214</v>
+      </c>
+      <c r="C28" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D28" s="30">
+        <v>400</v>
+      </c>
+      <c r="E28" s="30"/>
+      <c r="F28" s="30"/>
+      <c r="G28" s="30"/>
+      <c r="H28" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I28" s="30"/>
+      <c r="J28" s="30"/>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A29" s="30" t="s">
+        <v>220</v>
+      </c>
+      <c r="B29" s="30" t="s">
+        <v>218</v>
+      </c>
+      <c r="C29" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" s="30">
+        <v>400</v>
+      </c>
+      <c r="E29" s="30"/>
+      <c r="F29" s="30"/>
+      <c r="G29" s="30"/>
+      <c r="H29" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I29" s="30"/>
+      <c r="J29" s="30"/>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A30" s="30" t="s">
+        <v>223</v>
+      </c>
+      <c r="B30" s="30" t="s">
+        <v>221</v>
+      </c>
+      <c r="C30" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D30" s="30">
+        <v>400</v>
+      </c>
+      <c r="E30" s="30"/>
+      <c r="F30" s="30"/>
+      <c r="G30" s="30"/>
+      <c r="H30" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I30" s="30"/>
+      <c r="J30" s="30"/>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A31" s="30" t="s">
+        <v>226</v>
+      </c>
+      <c r="B31" s="30" t="s">
+        <v>224</v>
+      </c>
+      <c r="C31" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D31" s="30">
+        <v>200</v>
+      </c>
+      <c r="E31" s="30"/>
+      <c r="F31" s="30"/>
+      <c r="G31" s="30"/>
+      <c r="H31" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I31" s="30"/>
+      <c r="J31" s="30"/>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A32" s="30" t="s">
+        <v>230</v>
+      </c>
+      <c r="B32" s="30" t="s">
+        <v>227</v>
+      </c>
+      <c r="C32" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D32" s="30">
+        <v>400</v>
+      </c>
+      <c r="E32" s="30"/>
+      <c r="F32" s="30"/>
+      <c r="G32" s="30"/>
+      <c r="H32" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I32" s="30"/>
+      <c r="J32" s="30"/>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A33" s="30" t="s">
+        <v>233</v>
+      </c>
+      <c r="B33" s="30" t="s">
+        <v>231</v>
+      </c>
+      <c r="C33" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D33" s="30">
+        <v>400</v>
+      </c>
+      <c r="E33" s="30"/>
+      <c r="F33" s="30"/>
+      <c r="G33" s="30"/>
+      <c r="H33" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I33" s="30"/>
+      <c r="J33" s="30"/>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A34" s="30" t="s">
+        <v>236</v>
+      </c>
+      <c r="B34" s="30" t="s">
+        <v>234</v>
+      </c>
+      <c r="C34" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D34" s="30">
+        <v>400</v>
+      </c>
+      <c r="E34" s="30"/>
+      <c r="F34" s="30"/>
+      <c r="G34" s="30"/>
+      <c r="H34" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I34" s="30"/>
+      <c r="J34" s="30"/>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A35" s="30" t="s">
+        <v>238</v>
+      </c>
+      <c r="B35" s="30" t="s">
+        <v>237</v>
+      </c>
+      <c r="C35" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D35" s="30">
+        <v>400</v>
+      </c>
+      <c r="E35" s="30"/>
+      <c r="F35" s="30"/>
+      <c r="G35" s="30"/>
+      <c r="H35" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I35" s="30"/>
+      <c r="J35" s="30"/>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A36" s="30" t="s">
+        <v>241</v>
+      </c>
+      <c r="B36" s="30" t="s">
+        <v>239</v>
+      </c>
+      <c r="C36" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D36" s="30">
+        <v>400</v>
+      </c>
+      <c r="E36" s="30"/>
+      <c r="F36" s="30"/>
+      <c r="G36" s="30"/>
+      <c r="H36" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I36" s="30"/>
+      <c r="J36" s="30"/>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A37" s="30" t="s">
+        <v>243</v>
+      </c>
+      <c r="B37" s="30" t="s">
+        <v>242</v>
+      </c>
+      <c r="C37" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D37" s="30">
+        <v>400</v>
+      </c>
+      <c r="E37" s="30"/>
+      <c r="F37" s="30"/>
+      <c r="G37" s="30"/>
+      <c r="H37" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I37" s="30"/>
+      <c r="J37" s="30"/>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A38" s="30" t="s">
+        <v>272</v>
+      </c>
+      <c r="B38" s="30" t="s">
+        <v>284</v>
+      </c>
+      <c r="C38" s="30" t="s">
+        <v>14</v>
+      </c>
+      <c r="D38" s="30">
+        <v>200</v>
+      </c>
+      <c r="E38" s="30"/>
+      <c r="F38" s="30"/>
+      <c r="G38" s="30"/>
+      <c r="H38" s="30" t="s">
+        <v>19</v>
+      </c>
+      <c r="I38" s="30"/>
+      <c r="J38" s="30"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -3278,53 +4502,53 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="22" t="s">
         <v>210</v>
       </c>
-      <c r="B1" s="2"/>
+      <c r="B1" s="1"/>
     </row>
     <row r="2" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="B2" s="4">
-        <f>COUNTA(Product_TestCases!A3:A27)</f>
-        <v>25</v>
+      <c r="B2" s="3">
+        <f>COUNTA(Product_TestCases!A3:A44)</f>
+        <v>37</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="B3" s="6">
-        <f>COUNTIF(Product_TestCases!J3:J27,"High")</f>
-        <v>14</v>
+      <c r="B3" s="5">
+        <f>COUNTIF(Product_TestCases!J3:J44, "High")</f>
+        <v>24</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>74</v>
       </c>
-      <c r="B4" s="8">
-        <f>COUNTIF(Product_TestCases!J3:J27,"Medium")</f>
-        <v>9</v>
+      <c r="B4" s="7">
+        <f>COUNTIF(Product_TestCases!J3:J44,"Medium")</f>
+        <v>11</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="8" t="s">
         <v>148</v>
       </c>
-      <c r="B5" s="10">
-        <f>COUNTIF(Product_TestCases!J3:J27,"Low")</f>
+      <c r="B5" s="9">
+        <f>COUNTIF(Product_TestCases!J3:J44,"Low")</f>
         <v>2</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="B6" s="12">
-        <f>COUNTIF(Product_TestCases!K3:K27,"Pass")</f>
+      <c r="B6" s="11">
+        <f>COUNTIF(Product_TestCases!K3:K44,"Pass")</f>
         <v>0</v>
       </c>
     </row>
@@ -3332,44 +4556,44 @@
       <c r="A7" t="s">
         <v>76</v>
       </c>
-      <c r="B7" s="24">
-        <f>COUNTIF(Product_TestCases!K3:K27,"Fail")</f>
+      <c r="B7" s="23">
+        <f>COUNTIF(Product_TestCases!K3:K44,"Fail")</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A8" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="B8" s="14">
-        <f>COUNTIF(Product_TestCases!K3:K27,"Not Run")</f>
-        <v>25</v>
+      <c r="A8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="B8" s="13">
+        <f>COUNTIF(Product_TestCases!K3:K44,"Not Run")</f>
+        <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A9" s="15" t="s">
+      <c r="A9" s="14" t="s">
         <v>77</v>
       </c>
-      <c r="B9" s="16">
-        <f>COUNTIF(Product_TestCases!C3:C27,"POST")</f>
+      <c r="B9" s="15">
+        <f>COUNTIF(Product_TestCases!C3:C44,"POST")</f>
         <v>2</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A10" s="17" t="s">
+      <c r="A10" s="16" t="s">
         <v>78</v>
       </c>
-      <c r="B10" s="18">
-        <f>COUNTIF(Product_TestCases!C3:C27,"GET")</f>
-        <v>19</v>
+      <c r="B10" s="17">
+        <f>COUNTIF(Product_TestCases!C3:C44,"GET")</f>
+        <v>31</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="B11" s="20">
-        <f>COUNTIF(Product_TestCases!C3:C27,"PUT")</f>
+      <c r="B11" s="19">
+        <f>COUNTIF(Product_TestCases!C3:C44,"PUT")</f>
         <v>2</v>
       </c>
     </row>
@@ -3377,17 +4601,17 @@
       <c r="A12" t="s">
         <v>80</v>
       </c>
-      <c r="B12" s="24">
-        <f>COUNTIF(Product_TestCases!C3:C27,"DELETE")</f>
+      <c r="B12" s="23">
+        <f>COUNTIF(Product_TestCases!C3:C44,"DELETE")</f>
         <v>2</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A13" s="21" t="s">
+      <c r="A13" s="20" t="s">
         <v>81</v>
       </c>
-      <c r="B13" s="22">
-        <f>IF(COUNTA(Product_TestCases!A3:A27)&gt;0,(COUNTIF(Product_TestCases!K3:K27,"Pass")/COUNTA(Product_TestCases!A3:A27))*100,0)</f>
+      <c r="B13" s="21">
+        <f>IF(COUNTA(Product_TestCases!A3:A44)&gt;0,(COUNTIF(Product_TestCases!K3:K44,"Pass")/COUNTA(Product_TestCases!A3:A44))*100,0)</f>
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix Postman test assertions and duplicate name conflict for BVA cases
</commit_message>
<xml_diff>
--- a/automation/postman/VGA-store-product/VGA-store_product_AutoTest.xlsx
+++ b/automation/postman/VGA-store-product/VGA-store_product_AutoTest.xlsx
@@ -3919,7 +3919,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="H32" t="inlineStr">
         <is>
@@ -3969,7 +3969,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>400</v>
+        <v>200</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>

</xml_diff>